<commit_message>
chore(import): publish official import templates (#10)
Co-authored-by: Mokhtar Alsarori <msorori201201@gmail.com>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/import-templates/06_units_template.xlsx
+++ b/public/import-templates/06_units_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="41">
   <si>
     <t>unit_code *</t>
   </si>
@@ -29,6 +29,9 @@
     <t>sort_order</t>
   </si>
   <si>
+    <t>semester</t>
+  </si>
+  <si>
     <t>is_free</t>
   </si>
   <si>
@@ -108,6 +111,9 @@
   </si>
   <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>1 أو 2</t>
   </si>
   <si>
     <t>TRUE/FALSE</t>
@@ -521,17 +527,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="6" width="14" customWidth="1"/>
+    <col min="5" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -550,49 +556,58 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
-      <c r="F3" t="s">
-        <v>10</v>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -600,7 +615,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -611,29 +626,29 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -641,65 +656,65 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -707,13 +722,13 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -721,13 +736,13 @@
         <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -735,43 +750,57 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>